<commit_message>
update frcore deps cc7ea0172161927801fad48f4533b1c2021eb662
</commit_message>
<xml_diff>
--- a/nr-update-missing-fields/ig/StructureDefinition-as-dp-practitioner.xlsx
+++ b/nr-update-missing-fields/ig/StructureDefinition-as-dp-practitioner.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11058" uniqueCount="979">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11062" uniqueCount="981">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-17T12:12:47+00:00</t>
+    <t>2024-07-17T15:12:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2538,7 +2538,7 @@
     <t>The official certifications, training, and licenses that authorize or otherwise pertain to the provision of care by the practitioner.  For example, a medical license issued by a medical board authorizing the practitioner to practice medicine within a certian locality.</t>
   </si>
   <si>
-    <t xml:space="preserve">pattern:$this}
+    <t xml:space="preserve">value:code}
 </t>
   </si>
   <si>
@@ -2598,7 +2598,10 @@
     <t>Coded representation of the qualification.</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J105-EnsembleDiplome-RASS/FHIR/JDV-J105-EnsembleDiplome-RASS</t>
+    <t>Specific qualification the practitioner has to provide a service.</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/ValueSet/v2-2.7-0360</t>
   </si>
   <si>
     <t>./Qualifications.Value</t>
@@ -2794,6 +2797,10 @@
     <t>Practitioner.qualification.code.coding</t>
   </si>
   <si>
+    <t xml:space="preserve">value:system}
+</t>
+  </si>
+  <si>
     <t>Practitioner.qualification:degree.code.coding:degreeType</t>
   </si>
   <si>
@@ -2804,6 +2811,9 @@
   </si>
   <si>
     <t>Practitioner.qualification:degree.code.coding:degree</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J105-EnsembleDiplome-RASS/FHIR/JDV-J105-EnsembleDiplome-RASS</t>
   </si>
   <si>
     <t>Practitioner.qualification:degree.code.text</t>
@@ -2892,10 +2902,6 @@
     <t>Practitioner.qualification:exercicePro.code.coding</t>
   </si>
   <si>
-    <t xml:space="preserve">value:system}
-</t>
-  </si>
-  <si>
     <t>Practitioner.qualification:exercicePro.code.coding:categorieProfession</t>
   </si>
   <si>
@@ -2947,7 +2953,7 @@
     <t>savoirFaire</t>
   </si>
   <si>
-    <t>savoirFaire : Prérogatives d'exercice d'un professionnel reconnues par une autorité d'enregistrement sur une période donnée de son exercice professionnel, par exemple les spécialités ordinales, etc.</t>
+    <t>savoirFAire : Prérogatives d'exercice d'un professionnel reconnues par une autorité d'enregistrement sur une période donnée de son exercice professionnel, par exemple les spécialités ordinales, etc.</t>
   </si>
   <si>
     <t>Practitioner.qualification:savoirFaire.id</t>
@@ -29340,11 +29346,13 @@
         <v>78</v>
       </c>
       <c r="X223" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="Y223" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="Y223" t="s" s="2">
+        <v>827</v>
+      </c>
       <c r="Z223" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="AA223" t="s" s="2">
         <v>78</v>
@@ -29386,7 +29394,7 @@
         <v>810</v>
       </c>
       <c r="AN223" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="AO223" t="s" s="2">
         <v>78</v>
@@ -29394,10 +29402,10 @@
     </row>
     <row r="224" hidden="true">
       <c r="A224" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="B224" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C224" s="2"/>
       <c r="D224" t="s" s="2">
@@ -29423,14 +29431,14 @@
         <v>253</v>
       </c>
       <c r="L224" t="s" s="2">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="M224" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="N224" s="2"/>
       <c r="O224" t="s" s="2">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="P224" t="s" s="2">
         <v>78</v>
@@ -29479,7 +29487,7 @@
         <v>78</v>
       </c>
       <c r="AF224" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="AG224" t="s" s="2">
         <v>79</v>
@@ -29500,10 +29508,10 @@
         <v>78</v>
       </c>
       <c r="AM224" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="AN224" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="AO224" t="s" s="2">
         <v>78</v>
@@ -29511,10 +29519,10 @@
     </row>
     <row r="225" hidden="true">
       <c r="A225" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B225" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C225" s="2"/>
       <c r="D225" t="s" s="2">
@@ -29540,10 +29548,10 @@
         <v>476</v>
       </c>
       <c r="L225" t="s" s="2">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="M225" t="s" s="2">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="N225" s="2"/>
       <c r="O225" s="2"/>
@@ -29594,7 +29602,7 @@
         <v>78</v>
       </c>
       <c r="AF225" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="AG225" t="s" s="2">
         <v>79</v>
@@ -29615,7 +29623,7 @@
         <v>78</v>
       </c>
       <c r="AM225" t="s" s="2">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="AN225" t="s" s="2">
         <v>78</v>
@@ -29626,13 +29634,13 @@
     </row>
     <row r="226" hidden="true">
       <c r="A226" t="s" s="2">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="B226" t="s" s="2">
         <v>804</v>
       </c>
       <c r="C226" t="s" s="2">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="D226" t="s" s="2">
         <v>78</v>
@@ -29657,7 +29665,7 @@
         <v>805</v>
       </c>
       <c r="L226" t="s" s="2">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="M226" t="s" s="2">
         <v>807</v>
@@ -29743,7 +29751,7 @@
     </row>
     <row r="227" hidden="true">
       <c r="A227" t="s" s="2">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="B227" t="s" s="2">
         <v>812</v>
@@ -29858,7 +29866,7 @@
     </row>
     <row r="228" hidden="true">
       <c r="A228" t="s" s="2">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="B228" t="s" s="2">
         <v>813</v>
@@ -29971,13 +29979,13 @@
     </row>
     <row r="229" hidden="true">
       <c r="A229" t="s" s="2">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B229" t="s" s="2">
         <v>813</v>
       </c>
       <c r="C229" t="s" s="2">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="D229" t="s" s="2">
         <v>78</v>
@@ -29999,13 +30007,13 @@
         <v>78</v>
       </c>
       <c r="K229" t="s" s="2">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="L229" t="s" s="2">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="M229" t="s" s="2">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="N229" s="2"/>
       <c r="O229" s="2"/>
@@ -30088,10 +30096,10 @@
     </row>
     <row r="230" hidden="true">
       <c r="A230" t="s" s="2">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="B230" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C230" s="2"/>
       <c r="D230" t="s" s="2">
@@ -30203,10 +30211,10 @@
     </row>
     <row r="231" hidden="true">
       <c r="A231" t="s" s="2">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B231" t="s" s="2">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C231" s="2"/>
       <c r="D231" t="s" s="2">
@@ -30320,13 +30328,13 @@
     </row>
     <row r="232" hidden="true">
       <c r="A232" t="s" s="2">
+        <v>854</v>
+      </c>
+      <c r="B232" t="s" s="2">
         <v>853</v>
       </c>
-      <c r="B232" t="s" s="2">
-        <v>852</v>
-      </c>
       <c r="C232" t="s" s="2">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="D232" t="s" s="2">
         <v>78</v>
@@ -30437,10 +30445,10 @@
     </row>
     <row r="233" hidden="true">
       <c r="A233" t="s" s="2">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="B233" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C233" s="2"/>
       <c r="D233" t="s" s="2">
@@ -30552,10 +30560,10 @@
     </row>
     <row r="234" hidden="true">
       <c r="A234" t="s" s="2">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="B234" t="s" s="2">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C234" s="2"/>
       <c r="D234" t="s" s="2">
@@ -30667,10 +30675,10 @@
     </row>
     <row r="235" hidden="true">
       <c r="A235" t="s" s="2">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B235" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C235" s="2"/>
       <c r="D235" t="s" s="2">
@@ -30710,7 +30718,7 @@
       </c>
       <c r="Q235" s="2"/>
       <c r="R235" t="s" s="2">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="S235" t="s" s="2">
         <v>78</v>
@@ -30784,10 +30792,10 @@
     </row>
     <row r="236" hidden="true">
       <c r="A236" t="s" s="2">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B236" t="s" s="2">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C236" s="2"/>
       <c r="D236" t="s" s="2">
@@ -30847,7 +30855,7 @@
       </c>
       <c r="Y236" s="2"/>
       <c r="Z236" t="s" s="2">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="AA236" t="s" s="2">
         <v>78</v>
@@ -30897,13 +30905,13 @@
     </row>
     <row r="237" hidden="true">
       <c r="A237" t="s" s="2">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="B237" t="s" s="2">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C237" t="s" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="D237" t="s" s="2">
         <v>78</v>
@@ -31014,10 +31022,10 @@
     </row>
     <row r="238" hidden="true">
       <c r="A238" t="s" s="2">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="B238" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C238" s="2"/>
       <c r="D238" t="s" s="2">
@@ -31129,10 +31137,10 @@
     </row>
     <row r="239" hidden="true">
       <c r="A239" t="s" s="2">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B239" t="s" s="2">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C239" s="2"/>
       <c r="D239" t="s" s="2">
@@ -31244,10 +31252,10 @@
     </row>
     <row r="240" hidden="true">
       <c r="A240" t="s" s="2">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C240" s="2"/>
       <c r="D240" t="s" s="2">
@@ -31287,7 +31295,7 @@
       </c>
       <c r="Q240" s="2"/>
       <c r="R240" t="s" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="S240" t="s" s="2">
         <v>78</v>
@@ -31361,10 +31369,10 @@
     </row>
     <row r="241" hidden="true">
       <c r="A241" t="s" s="2">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C241" s="2"/>
       <c r="D241" t="s" s="2">
@@ -31424,7 +31432,7 @@
       </c>
       <c r="Y241" s="2"/>
       <c r="Z241" t="s" s="2">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="AA241" t="s" s="2">
         <v>78</v>
@@ -31474,13 +31482,13 @@
     </row>
     <row r="242" hidden="true">
       <c r="A242" t="s" s="2">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C242" t="s" s="2">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="D242" t="s" s="2">
         <v>78</v>
@@ -31591,10 +31599,10 @@
     </row>
     <row r="243" hidden="true">
       <c r="A243" t="s" s="2">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C243" s="2"/>
       <c r="D243" t="s" s="2">
@@ -31706,10 +31714,10 @@
     </row>
     <row r="244" hidden="true">
       <c r="A244" t="s" s="2">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B244" t="s" s="2">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C244" s="2"/>
       <c r="D244" t="s" s="2">
@@ -31821,10 +31829,10 @@
     </row>
     <row r="245" hidden="true">
       <c r="A245" t="s" s="2">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B245" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C245" s="2"/>
       <c r="D245" t="s" s="2">
@@ -31864,7 +31872,7 @@
       </c>
       <c r="Q245" s="2"/>
       <c r="R245" t="s" s="2">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="S245" t="s" s="2">
         <v>78</v>
@@ -31938,10 +31946,10 @@
     </row>
     <row r="246" hidden="true">
       <c r="A246" t="s" s="2">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B246" t="s" s="2">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C246" s="2"/>
       <c r="D246" t="s" s="2">
@@ -32001,7 +32009,7 @@
       </c>
       <c r="Y246" s="2"/>
       <c r="Z246" t="s" s="2">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="AA246" t="s" s="2">
         <v>78</v>
@@ -32051,10 +32059,10 @@
     </row>
     <row r="247" hidden="true">
       <c r="A247" t="s" s="2">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B247" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="C247" s="2"/>
       <c r="D247" t="s" s="2">
@@ -32094,7 +32102,7 @@
       </c>
       <c r="Q247" s="2"/>
       <c r="R247" t="s" s="2">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="S247" t="s" s="2">
         <v>78</v>
@@ -32168,10 +32176,10 @@
     </row>
     <row r="248" hidden="true">
       <c r="A248" t="s" s="2">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="B248" t="s" s="2">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C248" s="2"/>
       <c r="D248" t="s" s="2">
@@ -32283,7 +32291,7 @@
     </row>
     <row r="249" hidden="true">
       <c r="A249" t="s" s="2">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="B249" t="s" s="2">
         <v>814</v>
@@ -32402,7 +32410,7 @@
     </row>
     <row r="250" hidden="true">
       <c r="A250" t="s" s="2">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B250" t="s" s="2">
         <v>819</v>
@@ -32519,7 +32527,7 @@
     </row>
     <row r="251" hidden="true">
       <c r="A251" t="s" s="2">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="B251" t="s" s="2">
         <v>824</v>
@@ -32578,11 +32586,13 @@
         <v>78</v>
       </c>
       <c r="X251" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="Y251" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="Y251" t="s" s="2">
+        <v>827</v>
+      </c>
       <c r="Z251" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="AA251" t="s" s="2">
         <v>78</v>
@@ -32624,7 +32634,7 @@
         <v>810</v>
       </c>
       <c r="AN251" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="AO251" t="s" s="2">
         <v>78</v>
@@ -32632,10 +32642,10 @@
     </row>
     <row r="252" hidden="true">
       <c r="A252" t="s" s="2">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B252" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C252" s="2"/>
       <c r="D252" t="s" s="2">
@@ -32747,10 +32757,10 @@
     </row>
     <row r="253" hidden="true">
       <c r="A253" t="s" s="2">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="B253" t="s" s="2">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="C253" s="2"/>
       <c r="D253" t="s" s="2">
@@ -32841,7 +32851,7 @@
         <v>80</v>
       </c>
       <c r="AI253" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ253" t="s" s="2">
         <v>119</v>
@@ -32853,7 +32863,7 @@
         <v>78</v>
       </c>
       <c r="AM253" t="s" s="2">
-        <v>199</v>
+        <v>108</v>
       </c>
       <c r="AN253" t="s" s="2">
         <v>78</v>
@@ -32864,10 +32874,10 @@
     </row>
     <row r="254" hidden="true">
       <c r="A254" t="s" s="2">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B254" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C254" s="2"/>
       <c r="D254" t="s" s="2">
@@ -32939,7 +32949,7 @@
         <v>78</v>
       </c>
       <c r="AB254" t="s" s="2">
-        <v>808</v>
+        <v>893</v>
       </c>
       <c r="AC254" s="2"/>
       <c r="AD254" t="s" s="2">
@@ -32958,7 +32968,7 @@
         <v>80</v>
       </c>
       <c r="AI254" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ254" t="s" s="2">
         <v>102</v>
@@ -32981,13 +32991,13 @@
     </row>
     <row r="255" hidden="true">
       <c r="A255" t="s" s="2">
+        <v>894</v>
+      </c>
+      <c r="B255" t="s" s="2">
         <v>892</v>
       </c>
-      <c r="B255" t="s" s="2">
-        <v>891</v>
-      </c>
       <c r="C255" t="s" s="2">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="D255" t="s" s="2">
         <v>78</v>
@@ -33050,7 +33060,7 @@
       </c>
       <c r="Y255" s="2"/>
       <c r="Z255" t="s" s="2">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="AA255" t="s" s="2">
         <v>78</v>
@@ -33077,7 +33087,7 @@
         <v>80</v>
       </c>
       <c r="AI255" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ255" t="s" s="2">
         <v>102</v>
@@ -33100,13 +33110,13 @@
     </row>
     <row r="256" hidden="true">
       <c r="A256" t="s" s="2">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="B256" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C256" t="s" s="2">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="D256" t="s" s="2">
         <v>78</v>
@@ -33169,7 +33179,7 @@
       </c>
       <c r="Y256" s="2"/>
       <c r="Z256" t="s" s="2">
-        <v>827</v>
+        <v>898</v>
       </c>
       <c r="AA256" t="s" s="2">
         <v>78</v>
@@ -33196,7 +33206,7 @@
         <v>80</v>
       </c>
       <c r="AI256" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ256" t="s" s="2">
         <v>102</v>
@@ -33219,10 +33229,10 @@
     </row>
     <row r="257" hidden="true">
       <c r="A257" t="s" s="2">
-        <v>896</v>
+        <v>899</v>
       </c>
       <c r="B257" t="s" s="2">
-        <v>897</v>
+        <v>900</v>
       </c>
       <c r="C257" s="2"/>
       <c r="D257" t="s" s="2">
@@ -33315,7 +33325,7 @@
         <v>90</v>
       </c>
       <c r="AI257" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ257" t="s" s="2">
         <v>102</v>
@@ -33338,10 +33348,10 @@
     </row>
     <row r="258" hidden="true">
       <c r="A258" t="s" s="2">
-        <v>898</v>
+        <v>901</v>
       </c>
       <c r="B258" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C258" s="2"/>
       <c r="D258" t="s" s="2">
@@ -33367,14 +33377,14 @@
         <v>253</v>
       </c>
       <c r="L258" t="s" s="2">
-        <v>899</v>
+        <v>902</v>
       </c>
       <c r="M258" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="N258" s="2"/>
       <c r="O258" t="s" s="2">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="P258" t="s" s="2">
         <v>78</v>
@@ -33423,7 +33433,7 @@
         <v>78</v>
       </c>
       <c r="AF258" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="AG258" t="s" s="2">
         <v>79</v>
@@ -33444,10 +33454,10 @@
         <v>78</v>
       </c>
       <c r="AM258" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="AN258" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="AO258" t="s" s="2">
         <v>78</v>
@@ -33455,10 +33465,10 @@
     </row>
     <row r="259" hidden="true">
       <c r="A259" t="s" s="2">
-        <v>900</v>
+        <v>903</v>
       </c>
       <c r="B259" t="s" s="2">
-        <v>901</v>
+        <v>904</v>
       </c>
       <c r="C259" s="2"/>
       <c r="D259" t="s" s="2">
@@ -33570,10 +33580,10 @@
     </row>
     <row r="260" hidden="true">
       <c r="A260" t="s" s="2">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="B260" t="s" s="2">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="C260" s="2"/>
       <c r="D260" t="s" s="2">
@@ -33687,10 +33697,10 @@
     </row>
     <row r="261" hidden="true">
       <c r="A261" t="s" s="2">
-        <v>904</v>
+        <v>907</v>
       </c>
       <c r="B261" t="s" s="2">
-        <v>905</v>
+        <v>908</v>
       </c>
       <c r="C261" s="2"/>
       <c r="D261" t="s" s="2">
@@ -33716,7 +33726,7 @@
         <v>260</v>
       </c>
       <c r="L261" t="s" s="2">
-        <v>906</v>
+        <v>909</v>
       </c>
       <c r="M261" t="s" s="2">
         <v>262</v>
@@ -33804,10 +33814,10 @@
     </row>
     <row r="262" hidden="true">
       <c r="A262" t="s" s="2">
-        <v>907</v>
+        <v>910</v>
       </c>
       <c r="B262" t="s" s="2">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="C262" s="2"/>
       <c r="D262" t="s" s="2">
@@ -33833,7 +33843,7 @@
         <v>260</v>
       </c>
       <c r="L262" t="s" s="2">
-        <v>909</v>
+        <v>912</v>
       </c>
       <c r="M262" t="s" s="2">
         <v>271</v>
@@ -33923,10 +33933,10 @@
     </row>
     <row r="263" hidden="true">
       <c r="A263" t="s" s="2">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="B263" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C263" s="2"/>
       <c r="D263" t="s" s="2">
@@ -33949,13 +33959,13 @@
         <v>78</v>
       </c>
       <c r="K263" t="s" s="2">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="L263" t="s" s="2">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="M263" t="s" s="2">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="N263" s="2"/>
       <c r="O263" s="2"/>
@@ -34006,7 +34016,7 @@
         <v>78</v>
       </c>
       <c r="AF263" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="AG263" t="s" s="2">
         <v>79</v>
@@ -34027,7 +34037,7 @@
         <v>78</v>
       </c>
       <c r="AM263" t="s" s="2">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="AN263" t="s" s="2">
         <v>78</v>
@@ -34038,13 +34048,13 @@
     </row>
     <row r="264" hidden="true">
       <c r="A264" t="s" s="2">
-        <v>913</v>
+        <v>916</v>
       </c>
       <c r="B264" t="s" s="2">
         <v>804</v>
       </c>
       <c r="C264" t="s" s="2">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="D264" t="s" s="2">
         <v>78</v>
@@ -34069,7 +34079,7 @@
         <v>805</v>
       </c>
       <c r="L264" t="s" s="2">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="M264" t="s" s="2">
         <v>807</v>
@@ -34155,7 +34165,7 @@
     </row>
     <row r="265" hidden="true">
       <c r="A265" t="s" s="2">
-        <v>916</v>
+        <v>919</v>
       </c>
       <c r="B265" t="s" s="2">
         <v>812</v>
@@ -34270,7 +34280,7 @@
     </row>
     <row r="266" hidden="true">
       <c r="A266" t="s" s="2">
-        <v>917</v>
+        <v>920</v>
       </c>
       <c r="B266" t="s" s="2">
         <v>813</v>
@@ -34387,7 +34397,7 @@
     </row>
     <row r="267" hidden="true">
       <c r="A267" t="s" s="2">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="B267" t="s" s="2">
         <v>814</v>
@@ -34506,7 +34516,7 @@
     </row>
     <row r="268" hidden="true">
       <c r="A268" t="s" s="2">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B268" t="s" s="2">
         <v>819</v>
@@ -34623,7 +34633,7 @@
     </row>
     <row r="269" hidden="true">
       <c r="A269" t="s" s="2">
-        <v>920</v>
+        <v>923</v>
       </c>
       <c r="B269" t="s" s="2">
         <v>824</v>
@@ -34682,11 +34692,13 @@
         <v>78</v>
       </c>
       <c r="X269" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="Y269" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="Y269" t="s" s="2">
+        <v>827</v>
+      </c>
       <c r="Z269" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="AA269" t="s" s="2">
         <v>78</v>
@@ -34728,7 +34740,7 @@
         <v>810</v>
       </c>
       <c r="AN269" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="AO269" t="s" s="2">
         <v>78</v>
@@ -34736,10 +34748,10 @@
     </row>
     <row r="270" hidden="true">
       <c r="A270" t="s" s="2">
-        <v>921</v>
+        <v>924</v>
       </c>
       <c r="B270" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C270" s="2"/>
       <c r="D270" t="s" s="2">
@@ -34851,10 +34863,10 @@
     </row>
     <row r="271" hidden="true">
       <c r="A271" t="s" s="2">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="B271" t="s" s="2">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="C271" s="2"/>
       <c r="D271" t="s" s="2">
@@ -34945,7 +34957,7 @@
         <v>80</v>
       </c>
       <c r="AI271" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ271" t="s" s="2">
         <v>119</v>
@@ -34957,7 +34969,7 @@
         <v>78</v>
       </c>
       <c r="AM271" t="s" s="2">
-        <v>199</v>
+        <v>108</v>
       </c>
       <c r="AN271" t="s" s="2">
         <v>78</v>
@@ -34968,10 +34980,10 @@
     </row>
     <row r="272" hidden="true">
       <c r="A272" t="s" s="2">
-        <v>923</v>
+        <v>926</v>
       </c>
       <c r="B272" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C272" s="2"/>
       <c r="D272" t="s" s="2">
@@ -35043,7 +35055,7 @@
         <v>78</v>
       </c>
       <c r="AB272" t="s" s="2">
-        <v>924</v>
+        <v>893</v>
       </c>
       <c r="AC272" s="2"/>
       <c r="AD272" t="s" s="2">
@@ -35062,7 +35074,7 @@
         <v>80</v>
       </c>
       <c r="AI272" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ272" t="s" s="2">
         <v>102</v>
@@ -35085,13 +35097,13 @@
     </row>
     <row r="273" hidden="true">
       <c r="A273" t="s" s="2">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="B273" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C273" t="s" s="2">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="D273" t="s" s="2">
         <v>78</v>
@@ -35116,7 +35128,7 @@
         <v>154</v>
       </c>
       <c r="L273" t="s" s="2">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="M273" t="s" s="2">
         <v>395</v>
@@ -35154,7 +35166,7 @@
       </c>
       <c r="Y273" s="2"/>
       <c r="Z273" t="s" s="2">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="AA273" t="s" s="2">
         <v>78</v>
@@ -35181,7 +35193,7 @@
         <v>80</v>
       </c>
       <c r="AI273" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ273" t="s" s="2">
         <v>102</v>
@@ -35204,10 +35216,10 @@
     </row>
     <row r="274" hidden="true">
       <c r="A274" t="s" s="2">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="B274" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C274" t="s" s="2">
         <v>337</v>
@@ -35235,7 +35247,7 @@
         <v>154</v>
       </c>
       <c r="L274" t="s" s="2">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="M274" t="s" s="2">
         <v>395</v>
@@ -35300,7 +35312,7 @@
         <v>80</v>
       </c>
       <c r="AI274" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ274" t="s" s="2">
         <v>102</v>
@@ -35323,10 +35335,10 @@
     </row>
     <row r="275" hidden="true">
       <c r="A275" t="s" s="2">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="B275" t="s" s="2">
-        <v>897</v>
+        <v>900</v>
       </c>
       <c r="C275" s="2"/>
       <c r="D275" t="s" s="2">
@@ -35419,7 +35431,7 @@
         <v>90</v>
       </c>
       <c r="AI275" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ275" t="s" s="2">
         <v>102</v>
@@ -35442,10 +35454,10 @@
     </row>
     <row r="276" hidden="true">
       <c r="A276" t="s" s="2">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="B276" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C276" s="2"/>
       <c r="D276" t="s" s="2">
@@ -35471,14 +35483,14 @@
         <v>253</v>
       </c>
       <c r="L276" t="s" s="2">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="M276" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="N276" s="2"/>
       <c r="O276" t="s" s="2">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="P276" t="s" s="2">
         <v>78</v>
@@ -35527,7 +35539,7 @@
         <v>78</v>
       </c>
       <c r="AF276" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="AG276" t="s" s="2">
         <v>79</v>
@@ -35548,10 +35560,10 @@
         <v>78</v>
       </c>
       <c r="AM276" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="AN276" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="AO276" t="s" s="2">
         <v>78</v>
@@ -35559,10 +35571,10 @@
     </row>
     <row r="277" hidden="true">
       <c r="A277" t="s" s="2">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="B277" t="s" s="2">
-        <v>901</v>
+        <v>904</v>
       </c>
       <c r="C277" s="2"/>
       <c r="D277" t="s" s="2">
@@ -35674,10 +35686,10 @@
     </row>
     <row r="278" hidden="true">
       <c r="A278" t="s" s="2">
-        <v>934</v>
+        <v>936</v>
       </c>
       <c r="B278" t="s" s="2">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="C278" s="2"/>
       <c r="D278" t="s" s="2">
@@ -35791,10 +35803,10 @@
     </row>
     <row r="279" hidden="true">
       <c r="A279" t="s" s="2">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="B279" t="s" s="2">
-        <v>905</v>
+        <v>908</v>
       </c>
       <c r="C279" s="2"/>
       <c r="D279" t="s" s="2">
@@ -35820,7 +35832,7 @@
         <v>260</v>
       </c>
       <c r="L279" t="s" s="2">
-        <v>936</v>
+        <v>938</v>
       </c>
       <c r="M279" t="s" s="2">
         <v>262</v>
@@ -35908,10 +35920,10 @@
     </row>
     <row r="280" hidden="true">
       <c r="A280" t="s" s="2">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="B280" t="s" s="2">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="C280" s="2"/>
       <c r="D280" t="s" s="2">
@@ -35937,7 +35949,7 @@
         <v>260</v>
       </c>
       <c r="L280" t="s" s="2">
-        <v>938</v>
+        <v>940</v>
       </c>
       <c r="M280" t="s" s="2">
         <v>271</v>
@@ -36027,10 +36039,10 @@
     </row>
     <row r="281" hidden="true">
       <c r="A281" t="s" s="2">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="B281" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C281" s="2"/>
       <c r="D281" t="s" s="2">
@@ -36056,10 +36068,10 @@
         <v>476</v>
       </c>
       <c r="L281" t="s" s="2">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="M281" t="s" s="2">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="N281" s="2"/>
       <c r="O281" s="2"/>
@@ -36110,7 +36122,7 @@
         <v>78</v>
       </c>
       <c r="AF281" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="AG281" t="s" s="2">
         <v>79</v>
@@ -36131,7 +36143,7 @@
         <v>78</v>
       </c>
       <c r="AM281" t="s" s="2">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="AN281" t="s" s="2">
         <v>78</v>
@@ -36142,13 +36154,13 @@
     </row>
     <row r="282" hidden="true">
       <c r="A282" t="s" s="2">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="B282" t="s" s="2">
         <v>804</v>
       </c>
       <c r="C282" t="s" s="2">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D282" t="s" s="2">
         <v>78</v>
@@ -36173,7 +36185,7 @@
         <v>805</v>
       </c>
       <c r="L282" t="s" s="2">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="M282" t="s" s="2">
         <v>807</v>
@@ -36259,7 +36271,7 @@
     </row>
     <row r="283" hidden="true">
       <c r="A283" t="s" s="2">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="B283" t="s" s="2">
         <v>812</v>
@@ -36374,7 +36386,7 @@
     </row>
     <row r="284" hidden="true">
       <c r="A284" t="s" s="2">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="B284" t="s" s="2">
         <v>813</v>
@@ -36491,7 +36503,7 @@
     </row>
     <row r="285" hidden="true">
       <c r="A285" t="s" s="2">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="B285" t="s" s="2">
         <v>814</v>
@@ -36610,7 +36622,7 @@
     </row>
     <row r="286" hidden="true">
       <c r="A286" t="s" s="2">
-        <v>946</v>
+        <v>948</v>
       </c>
       <c r="B286" t="s" s="2">
         <v>819</v>
@@ -36727,7 +36739,7 @@
     </row>
     <row r="287" hidden="true">
       <c r="A287" t="s" s="2">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="B287" t="s" s="2">
         <v>824</v>
@@ -36786,11 +36798,13 @@
         <v>78</v>
       </c>
       <c r="X287" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="Y287" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="Y287" t="s" s="2">
+        <v>827</v>
+      </c>
       <c r="Z287" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="AA287" t="s" s="2">
         <v>78</v>
@@ -36823,7 +36837,7 @@
         <v>102</v>
       </c>
       <c r="AK287" t="s" s="2">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="AL287" t="s" s="2">
         <v>78</v>
@@ -36832,7 +36846,7 @@
         <v>810</v>
       </c>
       <c r="AN287" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="AO287" t="s" s="2">
         <v>78</v>
@@ -36840,10 +36854,10 @@
     </row>
     <row r="288" hidden="true">
       <c r="A288" t="s" s="2">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="B288" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C288" s="2"/>
       <c r="D288" t="s" s="2">
@@ -36955,10 +36969,10 @@
     </row>
     <row r="289" hidden="true">
       <c r="A289" t="s" s="2">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="B289" t="s" s="2">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="C289" s="2"/>
       <c r="D289" t="s" s="2">
@@ -37049,7 +37063,7 @@
         <v>80</v>
       </c>
       <c r="AI289" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ289" t="s" s="2">
         <v>119</v>
@@ -37061,7 +37075,7 @@
         <v>78</v>
       </c>
       <c r="AM289" t="s" s="2">
-        <v>199</v>
+        <v>108</v>
       </c>
       <c r="AN289" t="s" s="2">
         <v>78</v>
@@ -37072,10 +37086,10 @@
     </row>
     <row r="290" hidden="true">
       <c r="A290" t="s" s="2">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="B290" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C290" s="2"/>
       <c r="D290" t="s" s="2">
@@ -37147,7 +37161,7 @@
         <v>78</v>
       </c>
       <c r="AB290" t="s" s="2">
-        <v>924</v>
+        <v>893</v>
       </c>
       <c r="AC290" s="2"/>
       <c r="AD290" t="s" s="2">
@@ -37166,7 +37180,7 @@
         <v>80</v>
       </c>
       <c r="AI290" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ290" t="s" s="2">
         <v>102</v>
@@ -37189,13 +37203,13 @@
     </row>
     <row r="291" hidden="true">
       <c r="A291" t="s" s="2">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="B291" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C291" t="s" s="2">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="D291" t="s" s="2">
         <v>78</v>
@@ -37220,7 +37234,7 @@
         <v>154</v>
       </c>
       <c r="L291" t="s" s="2">
-        <v>954</v>
+        <v>956</v>
       </c>
       <c r="M291" t="s" s="2">
         <v>395</v>
@@ -37258,7 +37272,7 @@
       </c>
       <c r="Y291" s="2"/>
       <c r="Z291" t="s" s="2">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="AA291" t="s" s="2">
         <v>78</v>
@@ -37285,7 +37299,7 @@
         <v>80</v>
       </c>
       <c r="AI291" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ291" t="s" s="2">
         <v>102</v>
@@ -37308,13 +37322,13 @@
     </row>
     <row r="292" hidden="true">
       <c r="A292" t="s" s="2">
-        <v>956</v>
+        <v>958</v>
       </c>
       <c r="B292" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C292" t="s" s="2">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D292" t="s" s="2">
         <v>78</v>
@@ -37339,7 +37353,7 @@
         <v>154</v>
       </c>
       <c r="L292" t="s" s="2">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="M292" t="s" s="2">
         <v>395</v>
@@ -37377,7 +37391,7 @@
       </c>
       <c r="Y292" s="2"/>
       <c r="Z292" t="s" s="2">
-        <v>958</v>
+        <v>960</v>
       </c>
       <c r="AA292" t="s" s="2">
         <v>78</v>
@@ -37404,7 +37418,7 @@
         <v>80</v>
       </c>
       <c r="AI292" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ292" t="s" s="2">
         <v>102</v>
@@ -37427,10 +37441,10 @@
     </row>
     <row r="293" hidden="true">
       <c r="A293" t="s" s="2">
-        <v>959</v>
+        <v>961</v>
       </c>
       <c r="B293" t="s" s="2">
-        <v>897</v>
+        <v>900</v>
       </c>
       <c r="C293" s="2"/>
       <c r="D293" t="s" s="2">
@@ -37523,7 +37537,7 @@
         <v>90</v>
       </c>
       <c r="AI293" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ293" t="s" s="2">
         <v>102</v>
@@ -37546,10 +37560,10 @@
     </row>
     <row r="294" hidden="true">
       <c r="A294" t="s" s="2">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="B294" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C294" s="2"/>
       <c r="D294" t="s" s="2">
@@ -37575,14 +37589,14 @@
         <v>253</v>
       </c>
       <c r="L294" t="s" s="2">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="M294" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="N294" s="2"/>
       <c r="O294" t="s" s="2">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="P294" t="s" s="2">
         <v>78</v>
@@ -37631,7 +37645,7 @@
         <v>78</v>
       </c>
       <c r="AF294" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="AG294" t="s" s="2">
         <v>79</v>
@@ -37652,10 +37666,10 @@
         <v>78</v>
       </c>
       <c r="AM294" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="AN294" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="AO294" t="s" s="2">
         <v>78</v>
@@ -37663,10 +37677,10 @@
     </row>
     <row r="295" hidden="true">
       <c r="A295" t="s" s="2">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="B295" t="s" s="2">
-        <v>901</v>
+        <v>904</v>
       </c>
       <c r="C295" s="2"/>
       <c r="D295" t="s" s="2">
@@ -37778,10 +37792,10 @@
     </row>
     <row r="296" hidden="true">
       <c r="A296" t="s" s="2">
-        <v>962</v>
+        <v>964</v>
       </c>
       <c r="B296" t="s" s="2">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="C296" s="2"/>
       <c r="D296" t="s" s="2">
@@ -37895,10 +37909,10 @@
     </row>
     <row r="297" hidden="true">
       <c r="A297" t="s" s="2">
-        <v>963</v>
+        <v>965</v>
       </c>
       <c r="B297" t="s" s="2">
-        <v>905</v>
+        <v>908</v>
       </c>
       <c r="C297" s="2"/>
       <c r="D297" t="s" s="2">
@@ -37924,7 +37938,7 @@
         <v>260</v>
       </c>
       <c r="L297" t="s" s="2">
-        <v>964</v>
+        <v>966</v>
       </c>
       <c r="M297" t="s" s="2">
         <v>262</v>
@@ -37995,7 +38009,7 @@
         <v>102</v>
       </c>
       <c r="AK297" t="s" s="2">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="AL297" t="s" s="2">
         <v>266</v>
@@ -38012,10 +38026,10 @@
     </row>
     <row r="298" hidden="true">
       <c r="A298" t="s" s="2">
-        <v>966</v>
+        <v>968</v>
       </c>
       <c r="B298" t="s" s="2">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="C298" s="2"/>
       <c r="D298" t="s" s="2">
@@ -38041,7 +38055,7 @@
         <v>260</v>
       </c>
       <c r="L298" t="s" s="2">
-        <v>967</v>
+        <v>969</v>
       </c>
       <c r="M298" t="s" s="2">
         <v>271</v>
@@ -38114,7 +38128,7 @@
         <v>102</v>
       </c>
       <c r="AK298" t="s" s="2">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="AL298" t="s" s="2">
         <v>275</v>
@@ -38131,10 +38145,10 @@
     </row>
     <row r="299" hidden="true">
       <c r="A299" t="s" s="2">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="B299" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C299" s="2"/>
       <c r="D299" t="s" s="2">
@@ -38160,10 +38174,10 @@
         <v>476</v>
       </c>
       <c r="L299" t="s" s="2">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="M299" t="s" s="2">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="N299" s="2"/>
       <c r="O299" s="2"/>
@@ -38214,7 +38228,7 @@
         <v>78</v>
       </c>
       <c r="AF299" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="AG299" t="s" s="2">
         <v>79</v>
@@ -38235,7 +38249,7 @@
         <v>78</v>
       </c>
       <c r="AM299" t="s" s="2">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="AN299" t="s" s="2">
         <v>78</v>
@@ -38246,10 +38260,10 @@
     </row>
     <row r="300" hidden="true">
       <c r="A300" t="s" s="2">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="B300" t="s" s="2">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="C300" s="2"/>
       <c r="D300" t="s" s="2">
@@ -38272,19 +38286,19 @@
         <v>78</v>
       </c>
       <c r="K300" t="s" s="2">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="L300" t="s" s="2">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="M300" t="s" s="2">
-        <v>973</v>
+        <v>975</v>
       </c>
       <c r="N300" t="s" s="2">
-        <v>974</v>
+        <v>976</v>
       </c>
       <c r="O300" t="s" s="2">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="P300" t="s" s="2">
         <v>78</v>
@@ -38313,7 +38327,7 @@
       </c>
       <c r="Y300" s="2"/>
       <c r="Z300" t="s" s="2">
-        <v>976</v>
+        <v>978</v>
       </c>
       <c r="AA300" t="s" s="2">
         <v>78</v>
@@ -38331,7 +38345,7 @@
         <v>78</v>
       </c>
       <c r="AF300" t="s" s="2">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="AG300" t="s" s="2">
         <v>79</v>
@@ -38349,10 +38363,10 @@
         <v>78</v>
       </c>
       <c r="AL300" t="s" s="2">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="AM300" t="s" s="2">
-        <v>978</v>
+        <v>980</v>
       </c>
       <c r="AN300" t="s" s="2">
         <v>78</v>

</xml_diff>

<commit_message>
update dep fr core 19197f20ff65bca50fb43fec35f62d44efa5ba5c
</commit_message>
<xml_diff>
--- a/nr-update-missing-fields/ig/StructureDefinition-as-dp-practitioner.xlsx
+++ b/nr-update-missing-fields/ig/StructureDefinition-as-dp-practitioner.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-17T15:12:21+00:00</t>
+    <t>2024-07-25T07:49:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -28723,7 +28723,7 @@
         <v>80</v>
       </c>
       <c r="H218" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="I218" t="s" s="2">
         <v>78</v>
@@ -29653,7 +29653,7 @@
         <v>80</v>
       </c>
       <c r="H226" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="I226" t="s" s="2">
         <v>78</v>

</xml_diff>